<commit_message>
"abnormal data check" mode introduced
</commit_message>
<xml_diff>
--- a/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
+++ b/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
@@ -268,10 +268,10 @@
     <t>Search Condition Settings</t>
   </si>
   <si>
-    <t>Soft / Hard Delete</t>
-  </si>
-  <si>
-    <t>Soft / Hard Delete (internal value)</t>
+    <t>Process Type</t>
+  </si>
+  <si>
+    <t>Process Type (internal value)</t>
   </si>
   <si>
     <t>Related Table Process Pattern (internal value)</t>
@@ -1652,9 +1652,9 @@
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="Task ID" dataDxfId="35"/>
     <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB Connection ID" dataDxfId="34" dataCellStyle="標準 2"/>
-    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="Soft / Hard Delete" dataDxfId="33"/>
-    <tableColumn id="15" xr3:uid="{F58118F0-6716-6C42-853A-3FBAEE07F4E8}" name="Soft / Hard Delete (internal value)" dataDxfId="32">
-      <calculatedColumnFormula array="1">_xlfn.IFS(テーブル32[[#This Row],[Soft / Hard Delete]]="Soft Delete","SOFT_DELETE",テーブル32[[#This Row],[Soft / Hard Delete]]="Hard Delete","HARD_DELETE",TRUE,"")</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="Process Type" dataDxfId="33"/>
+    <tableColumn id="15" xr3:uid="{F58118F0-6716-6C42-853A-3FBAEE07F4E8}" name="Process Type (internal value)" dataDxfId="32">
+      <calculatedColumnFormula array="1">_xlfn.IFS(テーブル32[[#This Row],[Process Type]]="Soft Delete","SOFT_DELETE",テーブル32[[#This Row],[Process Type]]="Hard Delete","HARD_DELETE",テーブル32[[#This Row],[Process Type]]="Abnormal Data Check","ABNORMAL_DATA_CHECK",TRUE,"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="Table Name" dataDxfId="31" dataCellStyle="標準 2"/>
     <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="ID Column Name" dataDxfId="30" dataCellStyle="標準 2"/>
@@ -2405,7 +2405,7 @@
       <c r="A5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8" t="str" cm="1">
-        <f t="array" ref="D5">_xlfn.IFS(テーブル32[[#This Row],[Soft / Hard Delete]]="Soft Delete","SOFT_DELETE",テーブル32[[#This Row],[Soft / Hard Delete]]="Hard Delete","HARD_DELETE",TRUE,"")</f>
+        <f t="array" ref="D5">_xlfn.IFS(テーブル32[[#This Row],[Process Type]]="Soft Delete","SOFT_DELETE",テーブル32[[#This Row],[Process Type]]="Hard Delete","HARD_DELETE",テーブル32[[#This Row],[Process Type]]="Abnormal Data Check","ABNORMAL_DATA_CHECK",TRUE,"")</f>
         <v/>
       </c>
       <c r="E5" s="8"/>
@@ -2434,7 +2434,7 @@
   <phoneticPr fontId="1"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5" xr:uid="{8F6F98C1-595C-9F49-B250-21CD2634841D}">
-      <formula1>"Soft Delete,Hard Delete"</formula1>
+      <formula1>"Soft Delete,Hard Delete,Abnormal Data Check"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5 N5" xr:uid="{7B8B2790-6C59-604D-89F1-3BD24DE216A5}">
       <formula1>"quotes('),(none)"</formula1>

</xml_diff>

<commit_message>
housekeep-db: Search Condition Operator column added to Search Condition Settings
</commit_message>
<xml_diff>
--- a/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
+++ b/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
   <si>
     <t>value</t>
   </si>
@@ -291,6 +291,9 @@
   <si>
     <t>housekeep-db: 
 English version added</t>
+  </si>
+  <si>
+    <t>Search Condition Operator</t>
   </si>
 </sst>
 </file>
@@ -1673,11 +1676,12 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A4:D5" insertRow="1" totalsRowShown="0" headerRowDxfId="20">
-  <autoFilter ref="A4:D5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A4:E5" insertRow="1" totalsRowShown="0" headerRowDxfId="20">
+  <autoFilter ref="A4:E5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{0B02141A-0F5F-8849-982C-6C0A6A7BEE4F}" name="Task ID" dataDxfId="19" dataCellStyle="標準 2"/>
     <tableColumn id="12" xr3:uid="{69A08ECC-4076-9E48-8CE9-3FABB073CA81}" name="Search Condition Column Name" dataDxfId="18"/>
+    <tableColumn id="13" xr3:uid="{893B5EF9-F206-4F82-8561-C2C5A6776814}" name="Search Condition Operator" dataDxfId="18"/>
     <tableColumn id="2" xr3:uid="{511F37DB-74E3-394C-9204-B1C6CA623CD0}" name="Search Condition Column Literal Symbol" dataDxfId="17"/>
     <tableColumn id="3" xr3:uid="{2F474AF9-6428-D446-9D8C-0FEF2C86FE1D}" name="Search Condition Column Value" dataDxfId="16" dataCellStyle="標準 2"/>
   </tableColumns>
@@ -2466,56 +2470,65 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E1BEA4-8682-2D4B-83F3-E3D5D9773981}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.5" style="6" customWidth="1"/>
     <col min="2" max="2" width="23.83203125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="25.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1640625" style="6" customWidth="1"/>
-    <col min="5" max="16384" width="7.5" style="6"/>
+    <col min="3" max="3" width="22" style="6" customWidth="1"/>
+    <col min="4" max="4" width="25.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.1640625" style="6" customWidth="1"/>
+    <col min="6" max="16384" width="7.5" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="E4" s="28" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
-      <c r="D5" s="7"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D5" s="8"/>
+      <c r="E5" s="7"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
-      <c r="D6" s="7"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C6" xr:uid="{F3EDCD97-3DDD-0A4D-ACDF-687A95CDC907}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D6" xr:uid="{F3EDCD97-3DDD-0A4D-ACDF-687A95CDC907}">
       <formula1>"quotes('),(none)"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C6" xr:uid="{349A10D3-12BD-43FB-95FF-0264E64069F5}">
+      <formula1>"equal,not equal"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Date column now accepted as time expiration columns
</commit_message>
<xml_diff>
--- a/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
+++ b/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
@@ -184,7 +184,7 @@
     <t>Timestamp Column Data Type</t>
   </si>
   <si>
-    <t>Soft Delete: Update Timestamp Column Name</t>
+    <t>Soft Delete: Update Date / Timestamp Column Name</t>
   </si>
   <si>
     <t>Soft Delete: Update User ID Column Name</t>
@@ -214,7 +214,7 @@
     <t>Yosuke Tanaka</t>
   </si>
   <si>
-    <t>Expiration Check: Timestamp Column Name</t>
+    <t>Expiration Check: Date / Timestamp Column Name</t>
   </si>
   <si>
     <t>Expiration Check: Timestamp Column Data Type</t>
@@ -235,7 +235,7 @@
     <t>Soft Delete: Update User ID Column Literal Symbol</t>
   </si>
   <si>
-    <t>Soft Delete: Update Timestamp Column Name</t>
+    <t>Soft Delete: Update Date / Timestamp Column Name</t>
   </si>
   <si>
     <t>locale</t>
@@ -1662,11 +1662,11 @@
     <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="Table Name" dataDxfId="31" dataCellStyle="標準 2"/>
     <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="ID Column Name" dataDxfId="30" dataCellStyle="標準 2"/>
     <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="ID Column Literal Symbol" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="Expiration Check: Timestamp Column Name" dataDxfId="28" dataCellStyle="標準 2"/>
+    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="Expiration Check: Date / Timestamp Column Name" dataDxfId="28" dataCellStyle="標準 2"/>
     <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="Expiration Check: Timestamp Column Data Type" dataDxfId="27"/>
     <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="Expiration Check: Validity Days" dataDxfId="26" dataCellStyle="標準 2"/>
     <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="Soft Delete Column Name" dataDxfId="25" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="24" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="Soft Delete: Update Date / Timestamp Column Name" dataDxfId="24" dataCellStyle="標準 2"/>
     <tableColumn id="9" xr3:uid="{0A6924E1-C0CB-AF40-A208-E0E96A257245}" name="Soft Delete: Update User ID Column Name" dataDxfId="23" dataCellStyle="標準 2"/>
     <tableColumn id="14" xr3:uid="{93BF3B4F-D2E8-A640-A768-A230439878D9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="22" dataCellStyle="標準 2"/>
     <tableColumn id="13" xr3:uid="{DE6ACC44-9137-0840-9711-E0D04FCC851F}" name="Soft Delete: Update User ID Column Value" dataDxfId="21" dataCellStyle="標準 2"/>
@@ -1703,7 +1703,7 @@
     <tableColumn id="3" xr3:uid="{59ED585B-1BCF-DB41-A333-2655E74C710D}" name="Related Table ID Column Name" dataDxfId="8" dataCellStyle="標準 2"/>
     <tableColumn id="14" xr3:uid="{75144EA6-AFC2-3646-9A0E-DD4A2D917411}" name="Related Table ID Column Literal Symbol" dataDxfId="7" dataCellStyle="標準 2"/>
     <tableColumn id="4" xr3:uid="{684AF203-54CE-5A42-8441-2636BF604DAF}" name="Soft Delete Column Name" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{1D070257-74D6-6746-B460-ACB59A1770E6}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{1D070257-74D6-6746-B460-ACB59A1770E6}" name="Soft Delete: Update Date / Timestamp Column Name" dataDxfId="5"/>
     <tableColumn id="6" xr3:uid="{59287FEB-061F-B946-B814-312CDD2F482D}" name="Soft Delete: Update User ID Column Name" dataDxfId="4"/>
     <tableColumn id="7" xr3:uid="{E0734288-8DC3-C342-98A6-DBC50A55CEF9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="3"/>
     <tableColumn id="8" xr3:uid="{D5E8A958-B06D-554D-B183-49DD307AC86A}" name="Soft Delete: Update User ID Column Value" dataDxfId="2"/>

</xml_diff>

<commit_message>
Unneeded 'timestamp column data type' column in format excels removed
</commit_message>
<xml_diff>
--- a/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
+++ b/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
@@ -1650,9 +1650,9 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A4:O5" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
-  <autoFilter ref="A4:O5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A4:N5" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+  <autoFilter ref="A4:N5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="Task ID" dataDxfId="35"/>
     <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB Connection ID" dataDxfId="34" dataCellStyle="標準 2"/>
     <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="Process Type" dataDxfId="33"/>
@@ -1663,7 +1663,6 @@
     <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="ID Column Name" dataDxfId="30" dataCellStyle="標準 2"/>
     <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="ID Column Literal Symbol" dataDxfId="29"/>
     <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="Expiration Check: Date / Timestamp Column Name" dataDxfId="28" dataCellStyle="標準 2"/>
-    <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="Expiration Check: Timestamp Column Data Type" dataDxfId="27"/>
     <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="Expiration Check: Validity Days" dataDxfId="26" dataCellStyle="標準 2"/>
     <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="Soft Delete Column Name" dataDxfId="25" dataCellStyle="標準 2"/>
     <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="Soft Delete: Update Date / Timestamp Column Name" dataDxfId="24" dataCellStyle="標準 2"/>
@@ -2130,9 +2129,7 @@
       <c r="B1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>30</v>
-      </c>
+      <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
@@ -2141,18 +2138,14 @@
       <c r="B2" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="C2" s="10"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="10"/>
       <c r="B3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>19</v>
-      </c>
+      <c r="C3" s="10"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="10"/>
@@ -2316,7 +2309,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{789F72C4-22B4-0242-AA9D-05DCD1C7C1AF}">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.5" style="6" customWidth="1"/>
@@ -2325,23 +2318,23 @@
     <col min="4" max="4" width="25.6640625" style="6" hidden="1" customWidth="1"/>
     <col min="5" max="6" width="20.1640625" style="6" customWidth="1"/>
     <col min="7" max="7" width="25.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="38" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="40" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="44.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="34.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="33.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="44.83203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="33.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="7.5" style="6"/>
+    <col min="8" max="8" width="38" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="40" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="44.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="33.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="44.83203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="33.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="7.5" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>23</v>
       </c>
@@ -2349,16 +2342,15 @@
         <v>64</v>
       </c>
       <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="30" t="s">
+      <c r="J3" s="30" t="s">
         <v>65</v>
       </c>
+      <c r="K3" s="30"/>
       <c r="L3" s="30"/>
       <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="31"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N3" s="31"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
         <v>51</v>
       </c>
@@ -2384,28 +2376,25 @@
         <v>41</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="J4" s="23" t="s">
         <v>43</v>
       </c>
+      <c r="J4" s="24" t="s">
+        <v>44</v>
+      </c>
       <c r="K4" s="24" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L4" s="24" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M4" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="N4" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="O4" s="25" t="s">
+      <c r="N4" s="25" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8" t="str" cm="1">
@@ -2418,33 +2407,29 @@
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="N5" s="8"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M5" s="8"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="15"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:O3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:N3"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5" xr:uid="{8F6F98C1-595C-9F49-B250-21CD2634841D}">
       <formula1>"Soft Delete,Hard Delete,Abnormal Data Check"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5 N5" xr:uid="{7B8B2790-6C59-604D-89F1-3BD24DE216A5}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5 M5" xr:uid="{7B8B2790-6C59-604D-89F1-3BD24DE216A5}">
       <formula1>"quotes('),(none)"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5" xr:uid="{77C8DCE9-D337-B146-99D9-21A4944967AD}">
-      <formula1>"LocalDateTime,OffsetDateTime"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2460,7 +2445,7 @@
           <x14:formula1>
             <xm:f>dropdown!$B$2:$B$20</xm:f>
           </x14:formula1>
-          <xm:sqref>N6</xm:sqref>
+          <xm:sqref>M6</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>